<commit_message>
Historico_Cortes - siembra/append Jul-2026
</commit_message>
<xml_diff>
--- a/Tablas/Historico_Cortes.xlsx
+++ b/Tablas/Historico_Cortes.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -723,6 +723,258 @@
       </c>
       <c r="J8" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>401</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-18</v>
+      </c>
+      <c r="E9" t="n">
+        <v>81</v>
+      </c>
+      <c r="F9" t="n">
+        <v>61</v>
+      </c>
+      <c r="G9" t="n">
+        <v>62</v>
+      </c>
+      <c r="H9" t="n">
+        <v>88</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>47</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-61</v>
+      </c>
+      <c r="E10" t="n">
+        <v>60</v>
+      </c>
+      <c r="F10" t="n">
+        <v>46</v>
+      </c>
+      <c r="G10" t="n">
+        <v>33</v>
+      </c>
+      <c r="H10" t="n">
+        <v>89</v>
+      </c>
+      <c r="I10" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>295</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>54</v>
+      </c>
+      <c r="G11" t="n">
+        <v>50</v>
+      </c>
+      <c r="H11" t="n">
+        <v>92</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>67</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-47</v>
+      </c>
+      <c r="E12" t="n">
+        <v>78</v>
+      </c>
+      <c r="F12" t="n">
+        <v>54</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" t="n">
+        <v>98</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>262</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="n">
+        <v>74</v>
+      </c>
+      <c r="F13" t="n">
+        <v>39</v>
+      </c>
+      <c r="G13" t="n">
+        <v>56</v>
+      </c>
+      <c r="H13" t="n">
+        <v>57</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-41</v>
+      </c>
+      <c r="E14" t="n">
+        <v>88</v>
+      </c>
+      <c r="F14" t="n">
+        <v>43</v>
+      </c>
+      <c r="G14" t="n">
+        <v>73</v>
+      </c>
+      <c r="H14" t="n">
+        <v>92</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>425</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-16</v>
+      </c>
+      <c r="E15" t="n">
+        <v>75</v>
+      </c>
+      <c r="F15" t="n">
+        <v>31</v>
+      </c>
+      <c r="G15" t="n">
+        <v>56</v>
+      </c>
+      <c r="H15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I15" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -736,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E113"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3269,6 +3521,2234 @@
         <v>1</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>262</v>
+      </c>
+      <c r="E114" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Luminaria superior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>45</v>
+      </c>
+      <c r="E115" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior encendida de día</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>39</v>
+      </c>
+      <c r="E116" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Luminaria inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>23</v>
+      </c>
+      <c r="E117" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Columna en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>18</v>
+      </c>
+      <c r="E118" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Luminaria superior intermitente</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>7</v>
+      </c>
+      <c r="E119" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Tapa faltante/deteriorada</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>3</v>
+      </c>
+      <c r="E120" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Luminaria inferior intermitente</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>2</v>
+      </c>
+      <c r="E121" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Limpieza de luminaria</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>2</v>
+      </c>
+      <c r="E122" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Inconvenientes con intervenciones de arbolado</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>19</v>
+      </c>
+      <c r="E123" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Reparación de juegos/estaciones de ejercicio en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>5</v>
+      </c>
+      <c r="E124" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Árbol obstruye semáforo, cartel u otro elemento.</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>4</v>
+      </c>
+      <c r="E125" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>4</v>
+      </c>
+      <c r="E126" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Reparación de rejas, bancos, mesas y sillas en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>4</v>
+      </c>
+      <c r="E127" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Reparación o daño de caniles en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>3</v>
+      </c>
+      <c r="E128" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Reparación de senderos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Inconvenientes con las tareas de guardián de plaza</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>2</v>
+      </c>
+      <c r="E130" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Reparación de monumento/obra de arte en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Instalación de rejas en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Reparación de fuentes en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Reparación de bebederos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Bache en calle de asfalto</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>109</v>
+      </c>
+      <c r="E135" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Reparación/construcción de cordón</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>51</v>
+      </c>
+      <c r="E136" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Reparación de vereda por obra mal terminada</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>19</v>
+      </c>
+      <c r="E137" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Repavimentación de calle</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Bache en calle de hormigón</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Repintado / reparación de demarcación vial en calle o cordón</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>14</v>
+      </c>
+      <c r="E140" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Reparación de cuneta</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Construcción de cuneta</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Reparación de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>10</v>
+      </c>
+      <c r="E143" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Bache en calle de adoquines</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Construcción de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>6</v>
+      </c>
+      <c r="E145" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Inconvenientes con obras de bacheo</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>6</v>
+      </c>
+      <c r="E146" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Hidrolavado por grafitis/pegatinas</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>4</v>
+      </c>
+      <c r="E147" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Reparación de lomo de burro o reductor de velocidad</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo solicitud de limpieza</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Colocación de reductores de velocidad</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>3</v>
+      </c>
+      <c r="E151" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Estación de Metrobús en Mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo con riesgo de caída</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Reparación de elementos en túneles / puentes</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Retiro de afiches y/o pasacalles</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Parada de colectivo (poste) con Riesgo de caída</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Falta de Habilitación - Actividad no declarada</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>22</v>
+      </c>
+      <c r="E157" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Otros ruidos molestos</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>19</v>
+      </c>
+      <c r="E158" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Falta de higiene</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>8</v>
+      </c>
+      <c r="E159" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Música fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>6</v>
+      </c>
+      <c r="E160" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Venta de productos vencidos o en mal estado</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>4</v>
+      </c>
+      <c r="E161" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Obras fuera del horario permitido</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>2</v>
+      </c>
+      <c r="E162" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Ruidos molestos por aires acondicionados</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Carga y descarga fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>1</v>
+      </c>
+      <c r="E164" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Venta ambulante irregular</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Venta no habilitada de bebidas alcohólicas</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+      <c r="E166" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Ruidos Molestos por Autoelevadores</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Instalación eléctrica en mal estado/fuera de norma</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Cable cortado</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>115</v>
+      </c>
+      <c r="E169" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Roedores en espacio público</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>76</v>
+      </c>
+      <c r="E170" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Poste en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>15</v>
+      </c>
+      <c r="E171" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Reparación de vereda rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>10</v>
+      </c>
+      <c r="E172" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Agua servida en la vía pública proveniente de comercio o industria</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>8</v>
+      </c>
+      <c r="E173" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Ocupación irregular de objetos y/o vehículos</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>6</v>
+      </c>
+      <c r="E174" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Malos olores</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>5</v>
+      </c>
+      <c r="E175" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Poste quebrado/cortado</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>4</v>
+      </c>
+      <c r="E176" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Garita/puestos de diarios y/o flores irregulares</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>3</v>
+      </c>
+      <c r="E177" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Desobstrucción de cloacas</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>3</v>
+      </c>
+      <c r="E178" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Reparación de tapa de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>3</v>
+      </c>
+      <c r="E179" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Pasacalles en vía pública</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>3</v>
+      </c>
+      <c r="E180" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Otras plagas en espacio público</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>3</v>
+      </c>
+      <c r="E181" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Presencia de plagas /roedores, cucarachas…etc)</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>3</v>
+      </c>
+      <c r="E182" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Derrame tóxico o material riesgoso</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>2</v>
+      </c>
+      <c r="E183" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Nivelación de tapa de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Eventos irregulares en vía pública</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>1</v>
+      </c>
+      <c r="E185" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Reparación de calle rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Retiro de escombros y/o restos de obra</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>437</v>
+      </c>
+      <c r="E187" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o jardinería domiciliaria</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>270</v>
+      </c>
+      <c r="E188" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Falta de barrido o barrido deficiente</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>174</v>
+      </c>
+      <c r="E189" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Retiro de muebles y/o electrodomésticos en desuso</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>148</v>
+      </c>
+      <c r="E190" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Retiro de objetos/elementos en desuso</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>135</v>
+      </c>
+      <c r="E191" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos orgánicos/húmedos</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>115</v>
+      </c>
+      <c r="E192" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Limpieza/higienización de espacio público</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>38</v>
+      </c>
+      <c r="E193" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos reciclables (Programa Día Verde)</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>37</v>
+      </c>
+      <c r="E194" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o de arbolado público</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>27</v>
+      </c>
+      <c r="E195" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Vaciado de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>26</v>
+      </c>
+      <c r="E196" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Reposición de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>9</v>
+      </c>
+      <c r="E197" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Retiro de animales muertos en vía pública</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>8</v>
+      </c>
+      <c r="E198" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Reposición de contenedor</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>6</v>
+      </c>
+      <c r="E199" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Acopio de cartoneros en espacio público</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Colocación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>4</v>
+      </c>
+      <c r="E201" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas que interfieren en vía pública</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>4</v>
+      </c>
+      <c r="E202" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Irregularidades en la disposición de residuos húmedos/orgánicos</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>2</v>
+      </c>
+      <c r="E203" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Reparación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>2</v>
+      </c>
+      <c r="E204" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Personal de empresa de recolección con conductas indebidas</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>2</v>
+      </c>
+      <c r="E205" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Vaciado de contenedor</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>2</v>
+      </c>
+      <c r="E206" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Vehículos Abandonados</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>333</v>
+      </c>
+      <c r="E207" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Reparación de semáforo</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>66</v>
+      </c>
+      <c r="E208" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Vehículo mal estacionado</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Reparación de señal de tránsito</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>6</v>
+      </c>
+      <c r="E210" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Instalación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>4</v>
+      </c>
+      <c r="E211" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Reparación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>3</v>
+      </c>
+      <c r="E212" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Vehículo obstruyendo garage</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Historico_Cortes - siembra/append Ago-2026
</commit_message>
<xml_diff>
--- a/Tablas/Historico_Cortes.xlsx
+++ b/Tablas/Historico_Cortes.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -975,6 +975,258 @@
       </c>
       <c r="J15" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>565</v>
+      </c>
+      <c r="D16" t="n">
+        <v>42</v>
+      </c>
+      <c r="E16" t="n">
+        <v>89</v>
+      </c>
+      <c r="F16" t="n">
+        <v>62</v>
+      </c>
+      <c r="G16" t="n">
+        <v>72</v>
+      </c>
+      <c r="H16" t="n">
+        <v>91</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>98</v>
+      </c>
+      <c r="D17" t="n">
+        <v>123</v>
+      </c>
+      <c r="E17" t="n">
+        <v>49</v>
+      </c>
+      <c r="F17" t="n">
+        <v>77</v>
+      </c>
+      <c r="G17" t="n">
+        <v>54</v>
+      </c>
+      <c r="H17" t="n">
+        <v>92</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>405</v>
+      </c>
+      <c r="D18" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" t="n">
+        <v>31</v>
+      </c>
+      <c r="G18" t="n">
+        <v>44</v>
+      </c>
+      <c r="H18" t="n">
+        <v>74</v>
+      </c>
+      <c r="I18" t="n">
+        <v>9</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>101</v>
+      </c>
+      <c r="D19" t="n">
+        <v>55</v>
+      </c>
+      <c r="E19" t="n">
+        <v>78</v>
+      </c>
+      <c r="F19" t="n">
+        <v>52</v>
+      </c>
+      <c r="G19" t="n">
+        <v>33</v>
+      </c>
+      <c r="H19" t="n">
+        <v>96</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>275</v>
+      </c>
+      <c r="D20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>55</v>
+      </c>
+      <c r="F20" t="n">
+        <v>76</v>
+      </c>
+      <c r="G20" t="n">
+        <v>47</v>
+      </c>
+      <c r="H20" t="n">
+        <v>89</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1657</v>
+      </c>
+      <c r="D21" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" t="n">
+        <v>86</v>
+      </c>
+      <c r="F21" t="n">
+        <v>50</v>
+      </c>
+      <c r="G21" t="n">
+        <v>73</v>
+      </c>
+      <c r="H21" t="n">
+        <v>92</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>458</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" t="n">
+        <v>70</v>
+      </c>
+      <c r="F22" t="n">
+        <v>31</v>
+      </c>
+      <c r="G22" t="n">
+        <v>71</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -988,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5749,6 +6001,2418 @@
         <v>2</v>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>398</v>
+      </c>
+      <c r="E214" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Luminaria superior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>46</v>
+      </c>
+      <c r="E215" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Columna en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>34</v>
+      </c>
+      <c r="E216" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior encendida de día</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>33</v>
+      </c>
+      <c r="E217" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Luminaria inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>28</v>
+      </c>
+      <c r="E218" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Luminaria superior intermitente</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>17</v>
+      </c>
+      <c r="E219" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Tapa faltante/deteriorada</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>7</v>
+      </c>
+      <c r="E220" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Luminaria inferior intermitente</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>2</v>
+      </c>
+      <c r="E221" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Inconvenientes con intervenciones de arbolado</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>33</v>
+      </c>
+      <c r="E222" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>23</v>
+      </c>
+      <c r="E223" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Reparación de juegos/estaciones de ejercicio en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>7</v>
+      </c>
+      <c r="E224" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Reparación de bebederos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>7</v>
+      </c>
+      <c r="E225" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Árbol obstruye semáforo, cartel u otro elemento.</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>7</v>
+      </c>
+      <c r="E226" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Reparación de rejas, bancos, mesas y sillas en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>5</v>
+      </c>
+      <c r="E227" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Vaciado de cesto papelero en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>4</v>
+      </c>
+      <c r="E228" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Reparación o daño de caniles en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Reparación de senderos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Instalación de estaciones de ejercicio en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>1</v>
+      </c>
+      <c r="E231" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Construcción de senderos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>1</v>
+      </c>
+      <c r="E232" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Reparación de monumento/obra de arte en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Instalación de rejas en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E234" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Inconvenientes con las tareas de guardián de plaza</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Instalación de bebederos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Bache en calle de asfalto</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>178</v>
+      </c>
+      <c r="E237" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Reparación/construcción de cordón</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>76</v>
+      </c>
+      <c r="E238" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Bache en calle de hormigón</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>46</v>
+      </c>
+      <c r="E239" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Repavimentación de calle</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>20</v>
+      </c>
+      <c r="E240" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Reparación de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>15</v>
+      </c>
+      <c r="E241" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Repintado / reparación de demarcación vial en calle o cordón</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>10</v>
+      </c>
+      <c r="E242" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Construcción de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Reparación de cuneta</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo solicitud de limpieza</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>7</v>
+      </c>
+      <c r="E245" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Reparación de vereda por obra mal terminada</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>6</v>
+      </c>
+      <c r="E246" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Construcción de cuneta</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Reparación de rejas en esquina</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>5</v>
+      </c>
+      <c r="E248" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Bache en calle de adoquines</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Hidrolavado por grafitis/pegatinas</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>3</v>
+      </c>
+      <c r="E250" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Reparación de lomo de burro o reductor de velocidad</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>2</v>
+      </c>
+      <c r="E252" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Parada de colectivo (poste) en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>2</v>
+      </c>
+      <c r="E253" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Inconvenientes con obras de bacheo</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>2</v>
+      </c>
+      <c r="E254" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Reparación de elementos en túneles / puentes</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>2</v>
+      </c>
+      <c r="E255" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Estación de Metrobús en Mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo con riesgo de caída</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Estación de Metrobús solicitud de limpieza</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>1</v>
+      </c>
+      <c r="E258" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Falta de Habilitación - Actividad no declarada</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>37</v>
+      </c>
+      <c r="E259" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Otros ruidos molestos</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>25</v>
+      </c>
+      <c r="E260" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Falta de higiene</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>10</v>
+      </c>
+      <c r="E261" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Obras fuera del horario permitido</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>7</v>
+      </c>
+      <c r="E262" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Carga y descarga fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>5</v>
+      </c>
+      <c r="E263" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Ruidos molestos por aires acondicionados</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>4</v>
+      </c>
+      <c r="E264" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Venta de productos vencidos o en mal estado</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>3</v>
+      </c>
+      <c r="E265" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Actividad comercial fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>3</v>
+      </c>
+      <c r="E266" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Música fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>2</v>
+      </c>
+      <c r="E267" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Venta ambulante irregular</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>2</v>
+      </c>
+      <c r="E268" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Matafuegos faltantes y/o vencidos</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Ruidos Molestos por Autoelevadores</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Venta ilegal en vía pública</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>1</v>
+      </c>
+      <c r="E271" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Cable cortado</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>77</v>
+      </c>
+      <c r="E272" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Roedores en espacio público</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>77</v>
+      </c>
+      <c r="E273" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Poste en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>23</v>
+      </c>
+      <c r="E274" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Reparación de vereda rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>16</v>
+      </c>
+      <c r="E275" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Ocupación irregular de objetos y/o vehículos</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>16</v>
+      </c>
+      <c r="E276" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Agua servida en la vía pública proveniente de comercio o industria</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>12</v>
+      </c>
+      <c r="E277" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Malos olores</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>9</v>
+      </c>
+      <c r="E278" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Desobstrucción de cloacas</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>6</v>
+      </c>
+      <c r="E279" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Incon. En cámaras de inspec. de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>6</v>
+      </c>
+      <c r="E280" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Poste quebrado/cortado</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Abejas en espacio público</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>4</v>
+      </c>
+      <c r="E282" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Toldos/cerramientos/estructuras irregulares en vía pública</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>3</v>
+      </c>
+      <c r="E283" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Olores nauseabundos en vía pública</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Reparación de calle rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Otras plagas en espacio público</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>3</v>
+      </c>
+      <c r="E286" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Presencia de plagas /roedores, cucarachas…etc)</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>3</v>
+      </c>
+      <c r="E287" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Reparación de tapa de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>2</v>
+      </c>
+      <c r="E288" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Derrame tóxico o material riesgoso</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>2</v>
+      </c>
+      <c r="E289" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Reposición de tapa faltante de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Inconvenientes con el suministro de agua</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>1</v>
+      </c>
+      <c r="E291" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Pasacalles en vía pública</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>1</v>
+      </c>
+      <c r="E292" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Garita/puestos de diarios y/o flores irregulares</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Retiro de escombros y/o restos de obra</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>468</v>
+      </c>
+      <c r="E294" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o jardinería domiciliaria</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>321</v>
+      </c>
+      <c r="E295" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Retiro de objetos/elementos en desuso</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>221</v>
+      </c>
+      <c r="E296" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Retiro de muebles y/o electrodomésticos en desuso</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>165</v>
+      </c>
+      <c r="E297" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Falta de barrido o barrido deficiente</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>123</v>
+      </c>
+      <c r="E298" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos orgánicos/húmedos</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>116</v>
+      </c>
+      <c r="E299" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o de arbolado público</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>55</v>
+      </c>
+      <c r="E300" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos reciclables (Programa Día Verde)</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>52</v>
+      </c>
+      <c r="E301" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Limpieza/higienización de espacio público</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>39</v>
+      </c>
+      <c r="E302" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Vaciado de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>25</v>
+      </c>
+      <c r="E303" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas que interfieren en vía pública</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>16</v>
+      </c>
+      <c r="E304" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Colocación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>16</v>
+      </c>
+      <c r="E305" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Reposición de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>11</v>
+      </c>
+      <c r="E306" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Reposición de contenedor</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>7</v>
+      </c>
+      <c r="E307" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Acopio de cartoneros en espacio público</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Vaciado de contenedor</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>5</v>
+      </c>
+      <c r="E309" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Reparación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>4</v>
+      </c>
+      <c r="E310" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Retiro de animales muertos en vía pública</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>4</v>
+      </c>
+      <c r="E311" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Personal de empresa de recolección con conductas indebidas</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Irregularidades en la disposición de residuos húmedos/orgánicos</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>2</v>
+      </c>
+      <c r="E313" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Vehículos Abandonados</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>346</v>
+      </c>
+      <c r="E314" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Reparación de semáforo</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>66</v>
+      </c>
+      <c r="E315" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Vehículo mal estacionado</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Remoción de volquete abandonado o mal dispuesto</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Vehículo obstruyendo garage</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>6</v>
+      </c>
+      <c r="E318" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Reparación de señal de tránsito</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>4</v>
+      </c>
+      <c r="E319" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Instalación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>4</v>
+      </c>
+      <c r="E320" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Reparación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>